<commit_message>
Updated pulmonary shunting to distinguish between anatomic (with fluid mechanics changes) and physiologic (without fluid mechanics changes) by updating transport graph flows rather than circuit resistances. Other small validation updates.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/EnRouteCare/EnRouteCare.xlsx
+++ b/data/human/adult/validation/Scenarios/EnRouteCare/EnRouteCare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\EnRouteCare\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314FEBF7-6ECF-45E4-A243-5D6067C574F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63406A78-EC01-41A9-8E8E-D7B719E90F20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17550" yWindow="2805" windowWidth="37800" windowHeight="25620" tabRatio="500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29595" yWindow="3720" windowWidth="24480" windowHeight="25620" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patients" sheetId="8" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1384" uniqueCount="320">
   <si>
     <t>Scenario Name</t>
   </si>
@@ -1439,6 +1439,9 @@
   </si>
   <si>
     <t>{ "SerializeState": { "Mode": "Save", "Filename": "./states/EnRouteCare/Scenario7-InterventionApplied.json"} }</t>
+  </si>
+  <si>
+    <t>{ "SerializeState": { "Mode": "Save", "Filename": "./states/EnRouteCare/Scenario1-InsultsApplied.json"} }</t>
   </si>
 </sst>
 </file>
@@ -1957,10 +1960,28 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1982,24 +2003,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2795,7 +2798,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AMJ58"/>
+  <dimension ref="A1:AMJ59"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.85546875" style="11" customWidth="1"/>
@@ -2811,42 +2814,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1024" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
       <c r="AMG1" s="13"/>
       <c r="AMH1" s="13"/>
       <c r="AMI1" s="13"/>
       <c r="AMJ1" s="13"/>
     </row>
     <row r="2" spans="1:1024" ht="105.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
       <c r="E2" s="4" t="s">
         <v>286</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="47" t="s">
         <v>100</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
       <c r="AMG2" s="13"/>
       <c r="AMH2" s="13"/>
       <c r="AMI2" s="13"/>
@@ -2856,13 +2859,13 @@
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -2897,74 +2900,74 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:1024" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="52"/>
     </row>
     <row r="9" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="54"/>
     </row>
     <row r="10" spans="1:1024" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -3057,10 +3060,10 @@
       <c r="B16" s="39" t="s">
         <v>115</v>
       </c>
-      <c r="C16" s="52"/>
-      <c r="D16" s="52"/>
-      <c r="E16" s="52"/>
-      <c r="F16" s="53"/>
+      <c r="C16" s="41"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="41"/>
+      <c r="F16" s="42"/>
       <c r="G16" s="9" t="s">
         <v>114</v>
       </c>
@@ -3262,13 +3265,13 @@
       <c r="A26" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B26" s="41" t="s">
+      <c r="B26" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="41"/>
-      <c r="D26" s="41"/>
-      <c r="E26" s="41"/>
-      <c r="F26" s="41"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
       <c r="G26" s="1" t="s">
         <v>6</v>
       </c>
@@ -3338,12 +3341,12 @@
         <v>268</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="8">
         <v>2</v>
       </c>
       <c r="B31" s="39" t="s">
-        <v>98</v>
+        <v>319</v>
       </c>
       <c r="C31" s="39"/>
       <c r="D31" s="39"/>
@@ -3352,71 +3355,63 @@
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="6" t="s">
+    <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="8">
+        <v>2</v>
+      </c>
+      <c r="B32" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="C32" s="39"/>
+      <c r="D32" s="39"/>
+      <c r="E32" s="39"/>
+      <c r="F32" s="39"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A33" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B33" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C33" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E33" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="F33" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="G32" s="1" t="s">
+      <c r="G33" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H32" s="6" t="s">
+      <c r="H33" s="6" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="H33" s="17"/>
     </row>
     <row r="34" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="E34" s="10" t="s">
-        <v>70</v>
-      </c>
+        <v>191</v>
+      </c>
+      <c r="E34" s="10"/>
       <c r="F34" s="10"/>
-      <c r="G34" s="12" t="s">
-        <v>80</v>
+      <c r="G34" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="H34" s="17"/>
     </row>
@@ -3425,7 +3420,7 @@
         <v>27</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>39</v>
@@ -3438,7 +3433,7 @@
       </c>
       <c r="F35" s="10"/>
       <c r="G35" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H35" s="17"/>
     </row>
@@ -3447,20 +3442,20 @@
         <v>27</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="F36" s="10"/>
       <c r="G36" s="12" t="s">
-        <v>266</v>
+        <v>81</v>
       </c>
       <c r="H36" s="17"/>
     </row>
@@ -3469,20 +3464,20 @@
         <v>27</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>279</v>
+        <v>57</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="F37" s="10"/>
       <c r="G37" s="12" t="s">
-        <v>281</v>
+        <v>266</v>
       </c>
       <c r="H37" s="17"/>
     </row>
@@ -3491,20 +3486,20 @@
         <v>27</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>121</v>
+        <v>175</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>120</v>
+        <v>71</v>
       </c>
       <c r="F38" s="10"/>
-      <c r="G38" s="2" t="s">
-        <v>254</v>
+      <c r="G38" s="12" t="s">
+        <v>281</v>
       </c>
       <c r="H38" s="17"/>
     </row>
@@ -3513,324 +3508,324 @@
         <v>27</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>34</v>
+        <v>284</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>79</v>
+        <v>121</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>75</v>
+        <v>120</v>
       </c>
       <c r="F39" s="10"/>
       <c r="G39" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="H39" s="17"/>
+    </row>
+    <row r="40" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E40" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="F40" s="10"/>
+      <c r="G40" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="H39" s="17"/>
-    </row>
-    <row r="40" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="1" t="s">
+      <c r="H40" s="17"/>
+    </row>
+    <row r="41" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B40" s="41" t="s">
+      <c r="B41" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C40" s="41"/>
-      <c r="D40" s="41"/>
-      <c r="E40" s="41"/>
-      <c r="F40" s="41"/>
-      <c r="G40" s="1" t="s">
+      <c r="C41" s="40"/>
+      <c r="D41" s="40"/>
+      <c r="E41" s="40"/>
+      <c r="F41" s="40"/>
+      <c r="G41" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H40" s="6" t="s">
+      <c r="H41" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41" s="8">
-        <v>3</v>
-      </c>
-      <c r="B41" s="39" t="s">
-        <v>288</v>
-      </c>
-      <c r="C41" s="39"/>
-      <c r="D41" s="39"/>
-      <c r="E41" s="39"/>
-      <c r="F41" s="39"/>
-      <c r="G41" s="9"/>
-      <c r="H41" s="9"/>
-    </row>
-    <row r="42" spans="1:8" ht="263.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="8">
         <v>3</v>
       </c>
       <c r="B42" s="39" t="s">
-        <v>146</v>
-      </c>
-      <c r="C42" s="52"/>
-      <c r="D42" s="52"/>
-      <c r="E42" s="52"/>
-      <c r="F42" s="53"/>
-      <c r="G42" s="9" t="s">
-        <v>145</v>
-      </c>
-      <c r="H42" s="17"/>
-    </row>
-    <row r="43" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+        <v>288</v>
+      </c>
+      <c r="C42" s="39"/>
+      <c r="D42" s="39"/>
+      <c r="E42" s="39"/>
+      <c r="F42" s="39"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
+    </row>
+    <row r="43" spans="1:8" ht="263.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="8">
         <v>3</v>
       </c>
       <c r="B43" s="39" t="s">
+        <v>146</v>
+      </c>
+      <c r="C43" s="41"/>
+      <c r="D43" s="41"/>
+      <c r="E43" s="41"/>
+      <c r="F43" s="42"/>
+      <c r="G43" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="H43" s="17"/>
+    </row>
+    <row r="44" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="8">
+        <v>3</v>
+      </c>
+      <c r="B44" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="C43" s="39"/>
-      <c r="D43" s="39"/>
-      <c r="E43" s="39"/>
-      <c r="F43" s="39"/>
-      <c r="G43" s="9"/>
-      <c r="H43" s="17"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A44" s="6" t="s">
+      <c r="C44" s="39"/>
+      <c r="D44" s="39"/>
+      <c r="E44" s="39"/>
+      <c r="F44" s="39"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="17"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A45" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B44" s="6" t="s">
+      <c r="B45" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C45" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D44" s="1" t="s">
+      <c r="D45" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="E44" s="6" t="s">
+      <c r="E45" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="F45" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="G44" s="1" t="s">
+      <c r="G45" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H44" s="6" t="s">
+      <c r="H45" s="6" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="E45" s="10"/>
-      <c r="F45" s="10"/>
-      <c r="G45" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="H45" s="17"/>
     </row>
     <row r="46" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="E46" s="10" t="s">
-        <v>66</v>
-      </c>
+        <v>192</v>
+      </c>
+      <c r="E46" s="10"/>
       <c r="F46" s="10"/>
       <c r="G46" s="2" t="s">
-        <v>60</v>
+        <v>88</v>
       </c>
       <c r="H46" s="17"/>
     </row>
     <row r="47" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>284</v>
+        <v>33</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>193</v>
+        <v>168</v>
       </c>
       <c r="E47" s="10" t="s">
         <v>66</v>
       </c>
       <c r="F47" s="10"/>
       <c r="G47" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H47" s="17"/>
+    </row>
+    <row r="48" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="E48" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F48" s="10"/>
+      <c r="G48" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="H47" s="17"/>
-    </row>
-    <row r="48" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="1" t="s">
+      <c r="H48" s="17"/>
+    </row>
+    <row r="49" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B48" s="41" t="s">
+      <c r="B49" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="1" t="s">
+      <c r="C49" s="40"/>
+      <c r="D49" s="40"/>
+      <c r="E49" s="40"/>
+      <c r="F49" s="40"/>
+      <c r="G49" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H48" s="6" t="s">
+      <c r="H49" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="260.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="8">
-        <v>4</v>
-      </c>
-      <c r="B49" s="39" t="s">
-        <v>148</v>
-      </c>
-      <c r="C49" s="52"/>
-      <c r="D49" s="52"/>
-      <c r="E49" s="52"/>
-      <c r="F49" s="53"/>
-      <c r="G49" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="H49" s="17"/>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" ht="260.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="8">
         <v>4</v>
       </c>
       <c r="B50" s="39" t="s">
-        <v>289</v>
-      </c>
-      <c r="C50" s="39"/>
-      <c r="D50" s="39"/>
-      <c r="E50" s="39"/>
-      <c r="F50" s="39"/>
-      <c r="G50" s="9"/>
-      <c r="H50" s="9"/>
-    </row>
-    <row r="51" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+        <v>148</v>
+      </c>
+      <c r="C50" s="41"/>
+      <c r="D50" s="41"/>
+      <c r="E50" s="41"/>
+      <c r="F50" s="42"/>
+      <c r="G50" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="H50" s="17"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" s="8">
         <v>4</v>
       </c>
-      <c r="B51" s="54" t="s">
+      <c r="B51" s="39" t="s">
+        <v>289</v>
+      </c>
+      <c r="C51" s="39"/>
+      <c r="D51" s="39"/>
+      <c r="E51" s="39"/>
+      <c r="F51" s="39"/>
+      <c r="G51" s="9"/>
+      <c r="H51" s="9"/>
+    </row>
+    <row r="52" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="8">
+        <v>4</v>
+      </c>
+      <c r="B52" s="43" t="s">
         <v>69</v>
       </c>
-      <c r="C51" s="52"/>
-      <c r="D51" s="52"/>
-      <c r="E51" s="52"/>
-      <c r="F51" s="53"/>
-      <c r="G51" s="9"/>
-      <c r="H51" s="17"/>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A52" s="6" t="s">
+      <c r="C52" s="41"/>
+      <c r="D52" s="41"/>
+      <c r="E52" s="41"/>
+      <c r="F52" s="42"/>
+      <c r="G52" s="9"/>
+      <c r="H52" s="17"/>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A53" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B53" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C52" s="6" t="s">
+      <c r="C53" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D52" s="1" t="s">
+      <c r="D53" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="E52" s="6" t="s">
+      <c r="E53" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F52" s="1" t="s">
+      <c r="F53" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="G52" s="1" t="s">
+      <c r="G53" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H52" s="6" t="s">
+      <c r="H53" s="6" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="E53" s="10"/>
-      <c r="F53" s="10"/>
-      <c r="G53" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="H53" s="17"/>
     </row>
     <row r="54" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="E54" s="10" t="s">
-        <v>71</v>
-      </c>
+        <v>192</v>
+      </c>
+      <c r="E54" s="10"/>
       <c r="F54" s="10"/>
-      <c r="G54" s="12" t="s">
-        <v>56</v>
+      <c r="G54" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="H54" s="17"/>
     </row>
     <row r="55" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="F55" s="10"/>
-      <c r="G55" s="2" t="s">
-        <v>59</v>
+      <c r="G55" s="12" t="s">
+        <v>56</v>
       </c>
       <c r="H55" s="17"/>
     </row>
@@ -3839,29 +3834,29 @@
         <v>30</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F56" s="10"/>
       <c r="G56" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H56" s="17"/>
     </row>
     <row r="57" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>32</v>
@@ -3874,7 +3869,7 @@
       </c>
       <c r="F57" s="10"/>
       <c r="G57" s="2" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="H57" s="17"/>
     </row>
@@ -3883,52 +3878,48 @@
         <v>27</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>284</v>
+        <v>34</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>82</v>
       </c>
       <c r="F58" s="10"/>
       <c r="G58" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H58" s="17"/>
+    </row>
+    <row r="59" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="E59" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="F59" s="10"/>
+      <c r="G59" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="H58" s="17"/>
+      <c r="H59" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="37">
-    <mergeCell ref="B50:F50"/>
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="B51:F51"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B41:F41"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B42:F42"/>
-    <mergeCell ref="B43:F43"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="B29:F29"/>
+  <mergeCells count="38">
     <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B40:F40"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="G5:H5"/>
@@ -3939,6 +3930,33 @@
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="G6:H9"/>
     <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B51:F51"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B52:F52"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B41:F41"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3967,40 +3985,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1024" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
       <c r="AMI1" s="13"/>
       <c r="AMJ1" s="13"/>
     </row>
     <row r="2" spans="1:1024" ht="104.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
       <c r="E2" s="4" t="s">
         <v>290</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="47" t="s">
         <v>113</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
       <c r="AMI2" s="13"/>
       <c r="AMJ2" s="13"/>
     </row>
@@ -4008,13 +4026,13 @@
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -4049,14 +4067,14 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -4069,60 +4087,60 @@
         <v>16</v>
       </c>
       <c r="D6" s="7"/>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:1024" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="52"/>
     </row>
     <row r="9" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="54"/>
     </row>
     <row r="10" spans="1:1024" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -4380,13 +4398,13 @@
       <c r="A24" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B24" s="41" t="s">
+      <c r="B24" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="41"/>
-      <c r="D24" s="41"/>
-      <c r="E24" s="41"/>
-      <c r="F24" s="41"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
       <c r="G24" s="1" t="s">
         <v>6</v>
       </c>
@@ -4604,13 +4622,13 @@
       <c r="A36" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B36" s="41" t="s">
+      <c r="B36" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C36" s="41"/>
-      <c r="D36" s="41"/>
-      <c r="E36" s="41"/>
-      <c r="F36" s="41"/>
+      <c r="C36" s="40"/>
+      <c r="D36" s="40"/>
+      <c r="E36" s="40"/>
+      <c r="F36" s="40"/>
       <c r="G36" s="1" t="s">
         <v>6</v>
       </c>
@@ -4636,13 +4654,13 @@
       <c r="A38" s="8">
         <v>3</v>
       </c>
-      <c r="B38" s="54" t="s">
+      <c r="B38" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="C38" s="52"/>
-      <c r="D38" s="52"/>
-      <c r="E38" s="52"/>
-      <c r="F38" s="53"/>
+      <c r="C38" s="41"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="41"/>
+      <c r="F38" s="42"/>
       <c r="G38" s="9" t="s">
         <v>152</v>
       </c>
@@ -4812,27 +4830,6 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G6:H9"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="B38:F38"/>
@@ -4845,6 +4842,27 @@
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B37:F37"/>
     <mergeCell ref="B39:F39"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G6:H9"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -4873,50 +4891,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
       <c r="E2" s="4" t="s">
         <v>295</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="47" t="s">
         <v>112</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -4951,14 +4969,14 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -4971,60 +4989,60 @@
         <v>16</v>
       </c>
       <c r="D6" s="7"/>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="52"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="54"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="18" t="s">
         <v>6</v>
       </c>
@@ -5036,13 +5054,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="54" t="s">
+      <c r="B11" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="52"/>
-      <c r="D11" s="52"/>
-      <c r="E11" s="52"/>
-      <c r="F11" s="53"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="42"/>
       <c r="G11" s="19"/>
       <c r="H11" s="17" t="s">
         <v>22</v>
@@ -5052,13 +5070,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="54" t="s">
+      <c r="B12" s="43" t="s">
         <v>136</v>
       </c>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="53"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="42"/>
       <c r="G12" s="19"/>
       <c r="H12" s="17" t="s">
         <v>125</v>
@@ -5338,13 +5356,13 @@
       <c r="A27" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B27" s="41" t="s">
+      <c r="B27" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C27" s="41"/>
-      <c r="D27" s="41"/>
-      <c r="E27" s="41"/>
-      <c r="F27" s="41"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="40"/>
       <c r="G27" s="18" t="s">
         <v>6</v>
       </c>
@@ -11721,13 +11739,13 @@
       <c r="A42" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B42" s="41" t="s">
+      <c r="B42" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C42" s="41"/>
-      <c r="D42" s="41"/>
-      <c r="E42" s="41"/>
-      <c r="F42" s="41"/>
+      <c r="C42" s="40"/>
+      <c r="D42" s="40"/>
+      <c r="E42" s="40"/>
+      <c r="F42" s="40"/>
       <c r="G42" s="18" t="s">
         <v>6</v>
       </c>
@@ -15915,13 +15933,13 @@
       <c r="A49" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B49" s="41" t="s">
+      <c r="B49" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="41"/>
-      <c r="D49" s="41"/>
-      <c r="E49" s="41"/>
-      <c r="F49" s="41"/>
+      <c r="C49" s="40"/>
+      <c r="D49" s="40"/>
+      <c r="E49" s="40"/>
+      <c r="F49" s="40"/>
       <c r="G49" s="18" t="s">
         <v>6</v>
       </c>
@@ -20107,29 +20125,6 @@
     </row>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G6:H9"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B50:F50"/>
     <mergeCell ref="B52:F52"/>
     <mergeCell ref="B17:F17"/>
@@ -20146,6 +20141,29 @@
     <mergeCell ref="B45:F45"/>
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="B33:F33"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G6:H9"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -20174,50 +20192,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="154.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>128</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
       <c r="E2" s="4" t="s">
         <v>299</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="47" t="s">
         <v>111</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -20252,14 +20270,14 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -20272,60 +20290,60 @@
         <v>16</v>
       </c>
       <c r="D6" s="7"/>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="52"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="54"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -20353,13 +20371,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="54" t="s">
+      <c r="B12" s="43" t="s">
         <v>142</v>
       </c>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="53"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="42"/>
       <c r="G12" s="9"/>
       <c r="H12" s="17" t="s">
         <v>125</v>
@@ -20434,10 +20452,10 @@
       <c r="B17" s="39" t="s">
         <v>135</v>
       </c>
-      <c r="C17" s="52"/>
-      <c r="D17" s="52"/>
-      <c r="E17" s="52"/>
-      <c r="F17" s="53"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="42"/>
       <c r="G17" s="9" t="s">
         <v>134</v>
       </c>
@@ -20639,13 +20657,13 @@
       <c r="A27" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B27" s="41" t="s">
+      <c r="B27" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C27" s="41"/>
-      <c r="D27" s="41"/>
-      <c r="E27" s="41"/>
-      <c r="F27" s="41"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="40"/>
       <c r="G27" s="1" t="s">
         <v>6</v>
       </c>
@@ -20895,13 +20913,13 @@
       <c r="A40" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B40" s="41" t="s">
+      <c r="B40" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C40" s="41"/>
-      <c r="D40" s="41"/>
-      <c r="E40" s="41"/>
-      <c r="F40" s="41"/>
+      <c r="C40" s="40"/>
+      <c r="D40" s="40"/>
+      <c r="E40" s="40"/>
+      <c r="F40" s="40"/>
       <c r="G40" s="1" t="s">
         <v>6</v>
       </c>
@@ -21165,28 +21183,6 @@
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G6:H9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="B42:F42"/>
     <mergeCell ref="B45:F45"/>
@@ -21200,6 +21196,28 @@
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="B41:F41"/>
     <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G6:H9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -21228,50 +21246,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>250</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
       <c r="E2" s="4" t="s">
         <v>304</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="47" t="s">
         <v>110</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -21306,14 +21324,14 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -21326,60 +21344,60 @@
         <v>16</v>
       </c>
       <c r="D6" s="7"/>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="52"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="54"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -21456,10 +21474,10 @@
       <c r="B15" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="C15" s="52"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52"/>
-      <c r="F15" s="53"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="42"/>
       <c r="G15" s="9" t="s">
         <v>274</v>
       </c>
@@ -21661,13 +21679,13 @@
       <c r="A25" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B25" s="41" t="s">
+      <c r="B25" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C25" s="41"/>
-      <c r="D25" s="41"/>
-      <c r="E25" s="41"/>
-      <c r="F25" s="41"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
       <c r="G25" s="1" t="s">
         <v>6</v>
       </c>
@@ -21873,13 +21891,13 @@
       <c r="A36" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B36" s="41" t="s">
+      <c r="B36" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C36" s="41"/>
-      <c r="D36" s="41"/>
-      <c r="E36" s="41"/>
-      <c r="F36" s="41"/>
+      <c r="C36" s="40"/>
+      <c r="D36" s="40"/>
+      <c r="E36" s="40"/>
+      <c r="F36" s="40"/>
       <c r="G36" s="1" t="s">
         <v>6</v>
       </c>
@@ -22083,28 +22101,6 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G6:H9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="B38:F38"/>
-    <mergeCell ref="B13:F13"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B16:F16"/>
@@ -22115,6 +22111,28 @@
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B37:F37"/>
     <mergeCell ref="B39:F39"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G6:H9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -22143,50 +22161,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="160.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
       <c r="E2" s="4" t="s">
         <v>309</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="47" t="s">
         <v>109</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -22221,14 +22239,14 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -22241,60 +22259,60 @@
         <v>16</v>
       </c>
       <c r="D6" s="7"/>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="52"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="54"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -22368,13 +22386,13 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="54" t="s">
+      <c r="B15" s="43" t="s">
         <v>143</v>
       </c>
-      <c r="C15" s="52"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52"/>
-      <c r="F15" s="53"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="42"/>
       <c r="G15" s="9" t="s">
         <v>158</v>
       </c>
@@ -22556,13 +22574,13 @@
       <c r="A24" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B24" s="41" t="s">
+      <c r="B24" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="41"/>
-      <c r="D24" s="41"/>
-      <c r="E24" s="41"/>
-      <c r="F24" s="41"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
       <c r="G24" s="1" t="s">
         <v>6</v>
       </c>
@@ -22724,13 +22742,13 @@
       <c r="A33" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B33" s="41" t="s">
+      <c r="B33" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C33" s="41"/>
-      <c r="D33" s="41"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="40"/>
+      <c r="E33" s="40"/>
+      <c r="F33" s="40"/>
       <c r="G33" s="1" t="s">
         <v>6</v>
       </c>
@@ -22786,13 +22804,13 @@
       <c r="A37" s="8">
         <v>3</v>
       </c>
-      <c r="B37" s="54" t="s">
+      <c r="B37" s="43" t="s">
         <v>69</v>
       </c>
-      <c r="C37" s="52"/>
-      <c r="D37" s="52"/>
-      <c r="E37" s="52"/>
-      <c r="F37" s="53"/>
+      <c r="C37" s="41"/>
+      <c r="D37" s="41"/>
+      <c r="E37" s="41"/>
+      <c r="F37" s="42"/>
       <c r="G37" s="9" t="s">
         <v>119</v>
       </c>
@@ -22890,28 +22908,6 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G6:H9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B35:F35"/>
-    <mergeCell ref="B13:F13"/>
     <mergeCell ref="B37:F37"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B24:F24"/>
@@ -22922,6 +22918,28 @@
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B34:F34"/>
     <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G6:H9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -22950,50 +22968,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="40"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="49" t="s">
+      <c r="F1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="129" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
       <c r="E2" s="4" t="s">
         <v>314</v>
       </c>
-      <c r="F2" s="51" t="s">
+      <c r="F2" s="47" t="s">
         <v>105</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
@@ -23028,14 +23046,14 @@
       <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40" t="s">
+      <c r="F5" s="44"/>
+      <c r="G5" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="44"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -23048,60 +23066,60 @@
         <v>16</v>
       </c>
       <c r="D6" s="7"/>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="46"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="52"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="51"/>
+      <c r="H8" s="52"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="53"/>
+      <c r="H9" s="54"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -23129,13 +23147,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="54" t="s">
+      <c r="B12" s="43" t="s">
         <v>144</v>
       </c>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="53"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="42"/>
       <c r="G12" s="9"/>
       <c r="H12" s="17" t="s">
         <v>125</v>
@@ -23399,13 +23417,13 @@
       <c r="A26" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B26" s="41" t="s">
+      <c r="B26" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="41"/>
-      <c r="D26" s="41"/>
-      <c r="E26" s="41"/>
-      <c r="F26" s="41"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
       <c r="G26" s="1" t="s">
         <v>6</v>
       </c>
@@ -23567,13 +23585,13 @@
       <c r="A35" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B35" s="41" t="s">
+      <c r="B35" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="41"/>
-      <c r="D35" s="41"/>
-      <c r="E35" s="41"/>
-      <c r="F35" s="41"/>
+      <c r="C35" s="40"/>
+      <c r="D35" s="40"/>
+      <c r="E35" s="40"/>
+      <c r="F35" s="40"/>
       <c r="G35" s="1" t="s">
         <v>6</v>
       </c>
@@ -23733,28 +23751,6 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G6:H9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B35:F35"/>
     <mergeCell ref="B37:F37"/>
     <mergeCell ref="B39:F39"/>
@@ -23766,6 +23762,28 @@
     <mergeCell ref="B29:F29"/>
     <mergeCell ref="B36:F36"/>
     <mergeCell ref="B38:F38"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G6:H9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
En route care validation updates.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/EnRouteCare/EnRouteCare.xlsx
+++ b/data/human/adult/validation/Scenarios/EnRouteCare/EnRouteCare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\EnRouteCare\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD80A8A-3525-4575-AD00-3F2A7ABEB891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E098AA5-AD56-4B2E-9346-5F2FAD64565E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25635" yWindow="5070" windowWidth="27810" windowHeight="20550" tabRatio="500" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22050" yWindow="4575" windowWidth="27810" windowHeight="20550" tabRatio="500" firstSheet="8" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patients" sheetId="8" r:id="rId1"/>
@@ -1272,28 +1272,6 @@
  - High RR = 34 bpm (~10 bpm above the initial value or a max of 40 bpm)</t>
   </si>
   <si>
-    <t>Ventilator settings are:
-| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
-| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| VC-CMV | 0.650    | NA          | 70          | NA  | 0.6    | 14       | 5            | 0.4 |
-Ventilator alarm settings are:
- - High PIP = 40 cmH2O (~10 cmH2O above the initial value or a max of 40 cmH2O)
- - Low MVe = 6.8 L/min (~25% below the initial value)
- - Low VT = 490 mL (~25% below the initial value)
- - High RR = 24 bpm (~10 bpm above the initial value or a max of 40 bpm)</t>
-  </si>
-  <si>
-    <t>Ventilator settings are:
-| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
-| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| VC-CMV | 0.450  | NA          | 53           | NA  | 0.53  | 27       | 8            | 0.21 |
-Ventilator alarm settings are:
- - High PIP = 37 cmH2O (~10 cmH2O above the initial value or a max of 40 cmH2O)
- - Low MVe = 8.9 L/min (~25% below the initial value)
- - Low VT = 330 mL (~25% below the initial value)
- - High RR = 37 bpm (~10 bpm above the initial value or a max of 40 bpm)</t>
-  </si>
-  <si>
     <t>Ventilator settings are (VT Target = 6.9 mL/kg (ideal)):
 | Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
 | ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
@@ -1364,48 +1342,6 @@
   "RespirationRate": { "ScalarFrequency": { "Value": 24, "Unit": "1/min" } },
   "TidalVolume": { "ScalarVolume": { "Value": 490, "Unit": "mL" } },
   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
-    "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 40, "Unit": "cmH2O" } },
-    "HighPressureCycleOption": "On",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 6.8, "Unit": "L/min" } },
-    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 490, "Unit": "mL" } },
-    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 24, "Unit": "1/min" } } } } },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 70, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 14, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 650, "Unit": "mL" } },
-  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
-    "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 37, "Unit": "cmH2O" } },
-    "HighPressureCycleOption": "On",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 8.9, "Unit": "L/min" } },
-    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 330, "Unit": "mL" } },
-    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 37, "Unit": "1/min" } } } } },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 53, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.21 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.53, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 8, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 27, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 450, "Unit": "mL" } },
-   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
   }}
 }</t>
   </si>
@@ -1579,13 +1515,55 @@
     <t>{ "SerializeState": { "Mode": "Save", "Filename": "./states/EnRouteCare/Scenario7_NoSpontaneous-InterventionApplied.json"} }</t>
   </si>
   <si>
+    <t>{ "PatientAction": {
+      "AirwayObstruction": {
+        "Severity": {
+          "Scalar0To1": {
+            "Value": 0.4 } } ,
+         "HasSecretions": true } }
+  }</t>
+  </si>
+  <si>
+    <t>Ventilator settings are (VT Target = 6.6 mL/kg (ideal)):
+&lt;br /&gt;
+| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
+| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
+| VC-CMV | 0.376    | NA          | 42          | NA  | 0.6    | 26      | 5            | 0.4 |
+Ventilator alarm settings are:
+ - High PIP = 31 cmH2O (~10 cmH2O above the initial value or a max of 40 cmH2O)
+ - Low MVe = 7.3 L/min (~25% below the initial value)
+ - Low VT = 290 mL (~25% below the initial value)
+ - High RR = 36 bpm (~10 bpm above the initial value or a max of 40 bpm)</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
+    "SupplementalSettings": { "Alarms" : { 
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 31, "Unit": "cmH2O" } },
+    "HighPressureCycleOption": "On",
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 7.3, "Unit": "L/min" } },
+    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 290, "Unit": "mL" } },
+    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 36, "Unit": "1/min" } } } } },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 42, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 26, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 376, "Unit": "mL" } },
+  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
+  }}
+}</t>
+  </si>
+  <si>
     <t>Ventilator settings are:
 | Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
 | ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
 | PC-CMV | NA     | 25          | NA           | NA  | 0.6    | 10       | 34            | 0.60 |
 Ventilator alarm settings are:
- - High PIP = 30 cmH2O (~10 cmH2O above the initial value or a max of 40 cmH2O)
- - Low MVe = 11 L/min (~25% below the initial value)
+ - High PIP = 35 cmH2O (~10 cmH2O above the initial value or a max of 40 cmH2O)
+ - Low MVe = 9.6 L/min (~25% below the initial value)
  - Low VT = 310 mL (~25% below the initial value)
  - High RR = 40 bpm (~10 bpm above the initial value or a max of 40 bpm)</t>
   </si>
@@ -1593,9 +1571,9 @@
     <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
   { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
     "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 30, "Unit": "cmH2O" } },
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 35, "Unit": "cmH2O" } },
     "HighPressureCycleOption": "On",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 11, "Unit": "L/min" } },
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 9.6, "Unit": "L/min" } },
     "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 310, "Unit": "mL" } },
     "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 40, "Unit": "1/min" } } } } },
   "Mode": "AssistedControl", 
@@ -1615,8 +1593,8 @@
 | ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
 | PC-CMV | NA     | 18          | NA           | NA  | 0.8    | 23       | 5            | 0.40 |
 Ventilator alarm settings are:
- - High PIP = 24 cmH2O (~10 cmH2O above the initial value or a max of 40 cmH2O)
- - Low MVe = 8.4 L/min (~25% below the initial value)
+ - High PIP = 28 cmH2O (~10 cmH2O above the initial value or a max of 40 cmH2O)
+ - Low MVe = 7.9 L/min (~25% below the initial value)
  - Low VT = 365 mL (~25% below the initial value)
  - High RR = 33 bpm (~10 bpm above the initial value or a max of 40 bpm)</t>
   </si>
@@ -1624,9 +1602,9 @@
     <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
   { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
     "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 24, "Unit": "cmH2O" } },
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 28, "Unit": "cmH2O" } },
     "HighPressureCycleOption": "On",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 8.4, "Unit": "L/min" } },
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 7.9, "Unit": "L/min" } },
     "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 365, "Unit": "mL" } },
     "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 33, "Unit": "1/min" } } } } },
   "Mode": "AssistedControl", 
@@ -1641,46 +1619,68 @@
 }</t>
   </si>
   <si>
-    <t>Ventilator settings are (VT Target = 6.6 mL/kg (ideal)):
-&lt;br /&gt;
+    <t>Ventilator settings are:
 | Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
 | ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| VC-CMV | 0.376    | NA          | 42          | NA  | 0.6    | 26      | 5            | 0.4 |
+| VC-CMV | 0.650    | NA          | 70          | NA  | 0.6    | 14       | 5            | 0.4 |
 Ventilator alarm settings are:
- - High PIP = 26 cmH2O (~10 cmH2O above the initial value or a max of 40 cmH2O)
- - Low MVe = 7.5 L/min (~25% below the initial value)
- - Low VT = 290 mL (~25% below the initial value)
- - High RR = 36 bpm (~10 bpm above the initial value or a max of 40 bpm)</t>
+ - High PIP (no cycling) = 40 cmH2O (~10 cmH2O above the initial value or a max of 40 cmH2O)
+ - Low MVe = 6.8 L/min (~25% below the initial value)
+ - Low VT = 490 mL (~25% below the initial value)
+ - High RR = 24 bpm (~10 bpm above the initial value or a max of 40 bpm)</t>
   </si>
   <si>
     <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
   { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
     "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 26, "Unit": "cmH2O" } },
-    "HighPressureCycleOption": "On",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 7.5, "Unit": "L/min" } },
-    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 290, "Unit": "mL" } },
-    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 36, "Unit": "1/min" } } } } },
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 40, "Unit": "cmH2O" } },
+    "HighPressureCycleOption": "Off",
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 6.8, "Unit": "L/min" } },
+    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 490, "Unit": "mL" } },
+    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 24, "Unit": "1/min" } } } } },
   "Mode": "AssistedControl", 
   "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 42, "Unit": "L/min" } },
+  "Flow": { "ScalarVolumePerTime": { "Value": 70, "Unit": "L/min" } },
   "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
   "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
   "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 26, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 376, "Unit": "mL" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 14, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 650, "Unit": "mL" } },
   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
   }}
 }</t>
   </si>
   <si>
-    <t>{ "PatientAction": {
-      "AirwayObstruction": {
-        "Severity": {
-          "Scalar0To1": {
-            "Value": 0.4 } } ,
-         "HasSecretions": true } }
-  }</t>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
+    "SupplementalSettings": { "Alarms" : { 
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 37, "Unit": "cmH2O" } },
+    "HighPressureCycleOption": "Off",
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 8.9, "Unit": "L/min" } },
+    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 330, "Unit": "mL" } },
+    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 37, "Unit": "1/min" } } } } },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 53, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.21 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.53, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 8, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 27, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 450, "Unit": "mL" } },
+   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>Ventilator settings are:
+| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
+| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
+| VC-CMV | 0.450  | NA          | 53           | NA  | 0.53  | 27       | 8            | 0.21 |
+Ventilator alarm settings are:
+ - High PIP (no cycling) = 37 cmH2O (~10 cmH2O above the initial value or a max of 40 cmH2O)
+ - Low MVe = 8.9 L/min (~25% below the initial value)
+ - Low VT = 330 mL (~25% below the initial value)
+ - High RR = 37 bpm (~10 bpm above the initial value or a max of 40 bpm)</t>
   </si>
 </sst>
 </file>
@@ -3295,14 +3295,14 @@
         <v>1</v>
       </c>
       <c r="B16" s="39" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="C16" s="52"/>
       <c r="D16" s="52"/>
       <c r="E16" s="52"/>
       <c r="F16" s="53"/>
       <c r="G16" s="9" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="H16" s="17"/>
     </row>
@@ -3521,7 +3521,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="39" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="C27" s="39"/>
       <c r="D27" s="39"/>
@@ -3551,7 +3551,7 @@
         <v>2</v>
       </c>
       <c r="B29" s="39" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="C29" s="39"/>
       <c r="D29" s="39"/>
@@ -3733,7 +3733,7 @@
         <v>3</v>
       </c>
       <c r="B38" s="39" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="C38" s="39"/>
       <c r="D38" s="39"/>
@@ -3763,7 +3763,7 @@
         <v>3</v>
       </c>
       <c r="B40" s="39" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="C40" s="39"/>
       <c r="D40" s="39"/>
@@ -4211,7 +4211,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="54" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="C15" s="52"/>
       <c r="D15" s="52"/>
@@ -4431,7 +4431,7 @@
         <v>2</v>
       </c>
       <c r="B26" s="39" t="s">
-        <v>345</v>
+        <v>335</v>
       </c>
       <c r="C26" s="39"/>
       <c r="D26" s="39"/>
@@ -5034,14 +5034,14 @@
         <v>1</v>
       </c>
       <c r="B16" s="54" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C16" s="52"/>
       <c r="D16" s="52"/>
       <c r="E16" s="52"/>
       <c r="F16" s="53"/>
       <c r="G16" s="9" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="H16" s="17"/>
     </row>
@@ -5240,7 +5240,7 @@
         <v>2</v>
       </c>
       <c r="B26" s="39" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="C26" s="39"/>
       <c r="D26" s="39"/>
@@ -5254,7 +5254,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="39" t="s">
-        <v>345</v>
+        <v>335</v>
       </c>
       <c r="C27" s="39"/>
       <c r="D27" s="39"/>
@@ -5270,7 +5270,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
@@ -5408,7 +5408,7 @@
         <v>3</v>
       </c>
       <c r="B35" s="39" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C35" s="39"/>
       <c r="D35" s="39"/>
@@ -5438,7 +5438,7 @@
         <v>3</v>
       </c>
       <c r="B37" s="39" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="C37" s="39"/>
       <c r="D37" s="39"/>
@@ -5858,7 +5858,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="39" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="C16" s="39"/>
       <c r="D16" s="39"/>
@@ -6718,14 +6718,14 @@
         <v>1</v>
       </c>
       <c r="B17" s="39" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C17" s="39"/>
       <c r="D17" s="39"/>
       <c r="E17" s="39"/>
       <c r="F17" s="39"/>
       <c r="G17" s="9" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H17" s="17"/>
     </row>
@@ -6944,7 +6944,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
@@ -6974,7 +6974,7 @@
         <v>2</v>
       </c>
       <c r="B30" s="39" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="C30" s="39"/>
       <c r="D30" s="39"/>
@@ -7112,7 +7112,7 @@
         <v>3</v>
       </c>
       <c r="B37" s="39" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="C37" s="39"/>
       <c r="D37" s="39"/>
@@ -7142,7 +7142,7 @@
         <v>3</v>
       </c>
       <c r="B39" s="39" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="C39" s="39"/>
       <c r="D39" s="39"/>
@@ -7565,7 +7565,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="39" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C16" s="52"/>
       <c r="D16" s="52"/>
@@ -8091,7 +8091,7 @@
         <v>3</v>
       </c>
       <c r="B43" s="39" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C43" s="52"/>
       <c r="D43" s="52"/>
@@ -8229,7 +8229,7 @@
         <v>4</v>
       </c>
       <c r="B50" s="39" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C50" s="52"/>
       <c r="D50" s="52"/>
@@ -8736,7 +8736,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="39" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C16" s="52"/>
       <c r="D16" s="52"/>
@@ -8962,7 +8962,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="39" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="C27" s="39"/>
       <c r="D27" s="39"/>
@@ -9024,7 +9024,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="39" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="C31" s="39"/>
       <c r="D31" s="39"/>
@@ -9248,7 +9248,7 @@
         <v>3</v>
       </c>
       <c r="B42" s="39" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="C42" s="39"/>
       <c r="D42" s="39"/>
@@ -9262,7 +9262,7 @@
         <v>3</v>
       </c>
       <c r="B43" s="39" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C43" s="52"/>
       <c r="D43" s="52"/>
@@ -9400,7 +9400,7 @@
         <v>4</v>
       </c>
       <c r="B50" s="39" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C50" s="52"/>
       <c r="D50" s="52"/>
@@ -9416,7 +9416,7 @@
         <v>4</v>
       </c>
       <c r="B51" s="39" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="C51" s="39"/>
       <c r="D51" s="39"/>
@@ -9891,14 +9891,14 @@
         <v>1</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>310</v>
+        <v>343</v>
       </c>
       <c r="C15" s="39"/>
       <c r="D15" s="39"/>
       <c r="E15" s="39"/>
       <c r="F15" s="39"/>
       <c r="G15" s="9" t="s">
-        <v>304</v>
+        <v>342</v>
       </c>
       <c r="H15" s="17"/>
     </row>
@@ -10797,14 +10797,14 @@
         <v>1</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>310</v>
+        <v>343</v>
       </c>
       <c r="C15" s="39"/>
       <c r="D15" s="39"/>
       <c r="E15" s="39"/>
       <c r="F15" s="39"/>
       <c r="G15" s="9" t="s">
-        <v>304</v>
+        <v>342</v>
       </c>
       <c r="H15" s="17"/>
     </row>
@@ -11001,7 +11001,7 @@
         <v>2</v>
       </c>
       <c r="B25" s="39" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="C25" s="39"/>
       <c r="D25" s="39"/>
@@ -11045,7 +11045,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
@@ -11255,7 +11255,7 @@
         <v>3</v>
       </c>
       <c r="B39" s="39" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="C39" s="39"/>
       <c r="D39" s="39"/>
@@ -11733,14 +11733,14 @@
         <v>1</v>
       </c>
       <c r="B17" s="39" t="s">
-        <v>311</v>
+        <v>344</v>
       </c>
       <c r="C17" s="39"/>
       <c r="D17" s="39"/>
       <c r="E17" s="39"/>
       <c r="F17" s="39"/>
       <c r="G17" s="19" t="s">
-        <v>305</v>
+        <v>345</v>
       </c>
       <c r="H17" s="17"/>
     </row>
@@ -23552,7 +23552,7 @@
         <v>4</v>
       </c>
       <c r="B50" s="39" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C50" s="39"/>
       <c r="D50" s="39"/>
@@ -27034,14 +27034,14 @@
         <v>1</v>
       </c>
       <c r="B17" s="39" t="s">
-        <v>311</v>
+        <v>344</v>
       </c>
       <c r="C17" s="39"/>
       <c r="D17" s="39"/>
       <c r="E17" s="39"/>
       <c r="F17" s="39"/>
       <c r="G17" s="19" t="s">
-        <v>305</v>
+        <v>345</v>
       </c>
       <c r="H17" s="17"/>
     </row>
@@ -28276,7 +28276,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
@@ -34659,7 +34659,7 @@
         <v>3</v>
       </c>
       <c r="B43" s="39" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="C43" s="39"/>
       <c r="D43" s="39"/>
@@ -38853,7 +38853,7 @@
         <v>4</v>
       </c>
       <c r="B50" s="39" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C50" s="39"/>
       <c r="D50" s="39"/>
@@ -39885,7 +39885,7 @@
         <v>4</v>
       </c>
       <c r="B51" s="39" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="C51" s="39"/>
       <c r="D51" s="39"/>
@@ -42335,14 +42335,14 @@
         <v>1</v>
       </c>
       <c r="B17" s="39" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="C17" s="52"/>
       <c r="D17" s="52"/>
       <c r="E17" s="52"/>
       <c r="F17" s="53"/>
       <c r="G17" s="9" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H17" s="17"/>
     </row>
@@ -43357,7 +43357,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="C15" s="52"/>
       <c r="D15" s="52"/>

</xml_diff>

<commit_message>
Tweaked closed tension pneumothorax model to cause full collapse during positive pressure ventilation. Updated to en route care validation.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/EnRouteCare/EnRouteCare.xlsx
+++ b/data/human/adult/validation/Scenarios/EnRouteCare/EnRouteCare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\EnRouteCare\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E098AA5-AD56-4B2E-9346-5F2FAD64565E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B50026D-68E1-47DA-B672-31CB0CAE0CB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22050" yWindow="4575" windowWidth="27810" windowHeight="20550" tabRatio="500" firstSheet="8" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22050" yWindow="4575" windowWidth="27810" windowHeight="20550" tabRatio="500" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patients" sheetId="8" r:id="rId1"/>
@@ -1272,6 +1272,17 @@
  - High RR = 34 bpm (~10 bpm above the initial value or a max of 40 bpm)</t>
   </si>
   <si>
+    <t>Ventilator settings are:
+| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
+| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
+| VC-CMV | 0.450  | NA          | 53           | NA  | 0.53  | 27       | 8            | 0.21 |
+Ventilator alarm settings are:
+ - High PIP = 37 cmH2O (~10 cmH2O above the initial value or a max of 40 cmH2O)
+ - Low MVe = 8.9 L/min (~25% below the initial value)
+ - Low VT = 330 mL (~25% below the initial value)
+ - High RR = 37 bpm (~10 bpm above the initial value or a max of 40 bpm)</t>
+  </si>
+  <si>
     <t>Ventilator settings are (VT Target = 6.9 mL/kg (ideal)):
 | Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
 | ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
@@ -1342,6 +1353,27 @@
   "RespirationRate": { "ScalarFrequency": { "Value": 24, "Unit": "1/min" } },
   "TidalVolume": { "ScalarVolume": { "Value": 490, "Unit": "mL" } },
   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
+    "SupplementalSettings": { "Alarms" : { 
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 37, "Unit": "cmH2O" } },
+    "HighPressureCycleOption": "On",
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 8.9, "Unit": "L/min" } },
+    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 330, "Unit": "mL" } },
+    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 37, "Unit": "1/min" } } } } },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 53, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.21 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.53, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 8, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 27, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 450, "Unit": "mL" } },
+   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
   }}
 }</t>
   </si>
@@ -1649,38 +1681,6 @@
   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
   }}
 }</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
-    "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 37, "Unit": "cmH2O" } },
-    "HighPressureCycleOption": "Off",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 8.9, "Unit": "L/min" } },
-    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 330, "Unit": "mL" } },
-    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 37, "Unit": "1/min" } } } } },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 53, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.21 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.53, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 8, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 27, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 450, "Unit": "mL" } },
-   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>Ventilator settings are:
-| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
-| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| VC-CMV | 0.450  | NA          | 53           | NA  | 0.53  | 27       | 8            | 0.21 |
-Ventilator alarm settings are:
- - High PIP (no cycling) = 37 cmH2O (~10 cmH2O above the initial value or a max of 40 cmH2O)
- - Low MVe = 8.9 L/min (~25% below the initial value)
- - Low VT = 330 mL (~25% below the initial value)
- - High RR = 37 bpm (~10 bpm above the initial value or a max of 40 bpm)</t>
   </si>
 </sst>
 </file>
@@ -3295,14 +3295,14 @@
         <v>1</v>
       </c>
       <c r="B16" s="39" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C16" s="52"/>
       <c r="D16" s="52"/>
       <c r="E16" s="52"/>
       <c r="F16" s="53"/>
       <c r="G16" s="9" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="H16" s="17"/>
     </row>
@@ -3521,7 +3521,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="39" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="C27" s="39"/>
       <c r="D27" s="39"/>
@@ -3551,7 +3551,7 @@
         <v>2</v>
       </c>
       <c r="B29" s="39" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C29" s="39"/>
       <c r="D29" s="39"/>
@@ -3733,7 +3733,7 @@
         <v>3</v>
       </c>
       <c r="B38" s="39" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="C38" s="39"/>
       <c r="D38" s="39"/>
@@ -3763,7 +3763,7 @@
         <v>3</v>
       </c>
       <c r="B40" s="39" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C40" s="39"/>
       <c r="D40" s="39"/>
@@ -4211,7 +4211,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="54" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C15" s="52"/>
       <c r="D15" s="52"/>
@@ -4431,7 +4431,7 @@
         <v>2</v>
       </c>
       <c r="B26" s="39" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C26" s="39"/>
       <c r="D26" s="39"/>
@@ -5034,14 +5034,14 @@
         <v>1</v>
       </c>
       <c r="B16" s="54" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C16" s="52"/>
       <c r="D16" s="52"/>
       <c r="E16" s="52"/>
       <c r="F16" s="53"/>
       <c r="G16" s="9" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="H16" s="17"/>
     </row>
@@ -5240,7 +5240,7 @@
         <v>2</v>
       </c>
       <c r="B26" s="39" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C26" s="39"/>
       <c r="D26" s="39"/>
@@ -5254,7 +5254,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="39" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C27" s="39"/>
       <c r="D27" s="39"/>
@@ -5270,7 +5270,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
@@ -5408,7 +5408,7 @@
         <v>3</v>
       </c>
       <c r="B35" s="39" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C35" s="39"/>
       <c r="D35" s="39"/>
@@ -5438,7 +5438,7 @@
         <v>3</v>
       </c>
       <c r="B37" s="39" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C37" s="39"/>
       <c r="D37" s="39"/>
@@ -5858,7 +5858,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="39" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C16" s="39"/>
       <c r="D16" s="39"/>
@@ -6718,14 +6718,14 @@
         <v>1</v>
       </c>
       <c r="B17" s="39" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C17" s="39"/>
       <c r="D17" s="39"/>
       <c r="E17" s="39"/>
       <c r="F17" s="39"/>
       <c r="G17" s="9" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="H17" s="17"/>
     </row>
@@ -6944,7 +6944,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
@@ -6974,7 +6974,7 @@
         <v>2</v>
       </c>
       <c r="B30" s="39" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="C30" s="39"/>
       <c r="D30" s="39"/>
@@ -7112,7 +7112,7 @@
         <v>3</v>
       </c>
       <c r="B37" s="39" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C37" s="39"/>
       <c r="D37" s="39"/>
@@ -7142,7 +7142,7 @@
         <v>3</v>
       </c>
       <c r="B39" s="39" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="C39" s="39"/>
       <c r="D39" s="39"/>
@@ -7565,7 +7565,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="39" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C16" s="52"/>
       <c r="D16" s="52"/>
@@ -8091,7 +8091,7 @@
         <v>3</v>
       </c>
       <c r="B43" s="39" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C43" s="52"/>
       <c r="D43" s="52"/>
@@ -8229,7 +8229,7 @@
         <v>4</v>
       </c>
       <c r="B50" s="39" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C50" s="52"/>
       <c r="D50" s="52"/>
@@ -8736,7 +8736,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="39" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C16" s="52"/>
       <c r="D16" s="52"/>
@@ -8962,7 +8962,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="39" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C27" s="39"/>
       <c r="D27" s="39"/>
@@ -9024,7 +9024,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="39" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C31" s="39"/>
       <c r="D31" s="39"/>
@@ -9248,7 +9248,7 @@
         <v>3</v>
       </c>
       <c r="B42" s="39" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C42" s="39"/>
       <c r="D42" s="39"/>
@@ -9262,7 +9262,7 @@
         <v>3</v>
       </c>
       <c r="B43" s="39" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C43" s="52"/>
       <c r="D43" s="52"/>
@@ -9400,7 +9400,7 @@
         <v>4</v>
       </c>
       <c r="B50" s="39" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C50" s="52"/>
       <c r="D50" s="52"/>
@@ -9416,7 +9416,7 @@
         <v>4</v>
       </c>
       <c r="B51" s="39" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C51" s="39"/>
       <c r="D51" s="39"/>
@@ -9891,14 +9891,14 @@
         <v>1</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C15" s="39"/>
       <c r="D15" s="39"/>
       <c r="E15" s="39"/>
       <c r="F15" s="39"/>
       <c r="G15" s="9" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H15" s="17"/>
     </row>
@@ -10797,14 +10797,14 @@
         <v>1</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C15" s="39"/>
       <c r="D15" s="39"/>
       <c r="E15" s="39"/>
       <c r="F15" s="39"/>
       <c r="G15" s="9" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H15" s="17"/>
     </row>
@@ -11001,7 +11001,7 @@
         <v>2</v>
       </c>
       <c r="B25" s="39" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C25" s="39"/>
       <c r="D25" s="39"/>
@@ -11045,7 +11045,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
@@ -11255,7 +11255,7 @@
         <v>3</v>
       </c>
       <c r="B39" s="39" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C39" s="39"/>
       <c r="D39" s="39"/>
@@ -11733,14 +11733,14 @@
         <v>1</v>
       </c>
       <c r="B17" s="39" t="s">
-        <v>344</v>
+        <v>309</v>
       </c>
       <c r="C17" s="39"/>
       <c r="D17" s="39"/>
       <c r="E17" s="39"/>
       <c r="F17" s="39"/>
       <c r="G17" s="19" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="H17" s="17"/>
     </row>
@@ -23552,7 +23552,7 @@
         <v>4</v>
       </c>
       <c r="B50" s="39" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C50" s="39"/>
       <c r="D50" s="39"/>
@@ -27034,14 +27034,14 @@
         <v>1</v>
       </c>
       <c r="B17" s="39" t="s">
-        <v>344</v>
+        <v>309</v>
       </c>
       <c r="C17" s="39"/>
       <c r="D17" s="39"/>
       <c r="E17" s="39"/>
       <c r="F17" s="39"/>
       <c r="G17" s="19" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="H17" s="17"/>
     </row>
@@ -28276,7 +28276,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
@@ -34659,7 +34659,7 @@
         <v>3</v>
       </c>
       <c r="B43" s="39" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="C43" s="39"/>
       <c r="D43" s="39"/>
@@ -38853,7 +38853,7 @@
         <v>4</v>
       </c>
       <c r="B50" s="39" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C50" s="39"/>
       <c r="D50" s="39"/>
@@ -39885,7 +39885,7 @@
         <v>4</v>
       </c>
       <c r="B51" s="39" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C51" s="39"/>
       <c r="D51" s="39"/>
@@ -42335,14 +42335,14 @@
         <v>1</v>
       </c>
       <c r="B17" s="39" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C17" s="52"/>
       <c r="D17" s="52"/>
       <c r="E17" s="52"/>
       <c r="F17" s="53"/>
       <c r="G17" s="9" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="H17" s="17"/>
     </row>
@@ -43357,7 +43357,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C15" s="52"/>
       <c r="D15" s="52"/>

</xml_diff>

<commit_message>
Update scenarios with mechanical ventilator modes to have the connection in supplemental settings
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/EnRouteCare/EnRouteCare.xlsx
+++ b/data/human/adult/validation/Scenarios/EnRouteCare/EnRouteCare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\EnRouteCare\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Programming\Pulse\engine\data\human\adult\validation\Scenarios\EnRouteCare\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54E5426A-139B-4C32-BE42-A219C9CE0CD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{853751D1-EC21-4D2E-B0CF-73670D6CEB15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21960" yWindow="3855" windowWidth="28770" windowHeight="25050" tabRatio="500" firstSheet="9" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" firstSheet="9" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patients" sheetId="8" r:id="rId1"/>
@@ -934,68 +934,6 @@
  - None</t>
   </si>
   <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
-    "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 37, "Unit": "cmH2O" } },
-    "HighPressureCycleOption": "On",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 8.7, "Unit": "L/min" } },
-    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 360, "Unit": "mL" } },
-    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 34, "Unit": "1/min" } } } } },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 52, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 24, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 488, "Unit": "mL" } },
-  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
-    "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 26, "Unit": "cmH2O" } },
-    "HighPressureCycleOption": "On",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 7.5, "Unit": "L/min" } },
-    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 290, "Unit": "mL" } },
-    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 36, "Unit": "1/min" } } } } },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 42, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 12, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 376, "Unit": "mL" } },
-  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
-    "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 24, "Unit": "cmH2O" } },
-    "HighPressureCycleOption": "On",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 8.4, "Unit": "L/min" } },
-    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 365, "Unit": "mL" } },
-    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 33, "Unit": "1/min" } } } } },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.8, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 14.2, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 10, "Unit": "1/min" } },
-  "InspirationPatientTriggerFlow": { "ScalarVolumePerTime": { "Value": 1.0, "Unit": "L/min"  } }
-  }}
-}</t>
-  </si>
-  <si>
     <t>{ "SerializeState": { "Mode": "Save", "Filename": "./states/EnRouteCare/Scenario1_NoSpontaneous-InitialHemeostasis.json"} }</t>
   </si>
   <si>
@@ -1062,69 +1000,7 @@
     <t>{ "SerializeState": { "Mode": "Save", "Filename": "./states/EnRouteCare/Scenario7_NoSpontaneous-InterventionApplied.json"} }</t>
   </si>
   <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
-    "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 31, "Unit": "cmH2O" } },
-    "HighPressureCycleOption": "On",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 7.3, "Unit": "L/min" } },
-    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 290, "Unit": "mL" } },
-    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 36, "Unit": "1/min" } } } } },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 42, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 26, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 376, "Unit": "mL" } },
-  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
-    "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 28, "Unit": "cmH2O" } },
-    "HighPressureCycleOption": "On",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 7.9, "Unit": "L/min" } },
-    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 365, "Unit": "mL" } },
-    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 33, "Unit": "1/min" } } } } },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.8, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 18, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 23, "Unit": "1/min" } },
-  "InspirationPatientTriggerFlow": { "ScalarVolumePerTime": { "Value": 1.0, "Unit": "L/min"  } }
-  }}
-}</t>
-  </si>
-  <si>
     <t>{ "AdvanceTime": { "Time": { "ScalarTime": { "Value": 3, "Unit": "min" }}}}</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
-    "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 50, "Unit": "cmH2O" } },
-    "HighPressureCycleOption": "On",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 6.8, "Unit": "L/min" } },
-    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 490, "Unit": "mL" } },
-    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 24, "Unit": "1/min" } } } } },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 70, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 14, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 650, "Unit": "mL" } },
-  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
-  }}
-}</t>
   </si>
   <si>
     <t>VT for PIP alarm cycling</t>
@@ -1392,27 +1268,6 @@
  - SpO2, breath sounds, plateau pressure indicate pneumothorax resolved</t>
   </si>
   <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
-    "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 33, "Unit": "cmH2O" } },
-    "HighPressureCycleOption": "On",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 6.8, "Unit": "L/min" } },
-    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 330, "Unit": "mL" } },
-    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 30, "Unit": "1/min" } } } } },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 35, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.5 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.8, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 8, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 24, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 450, "Unit": "mL" } },
-   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
-  }}
-}</t>
-  </si>
-  <si>
     <t>{v} = 584</t>
   </si>
   <si>
@@ -1499,27 +1354,6 @@
  - Low MVe = 10.4 L/min (~25% below the initial value)
  - Low VT = 438 mL (~25% below the initial value)
  - High RR = 34 bpm (~10 bpm above the initial value or a max of 40 bpm)</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
-    "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 38, "Unit": "cmH2O" } },
-    "HighPressureCycleOption": "On",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 10.4, "Unit": "L/min" } },
-    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 438, "Unit": "mL" } },
-    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 34, "Unit": "1/min" } } } } },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 60, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.62, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 24, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 584, "Unit": "mL" } },
-  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
-  }}
-}</t>
   </si>
   <si>
     <t>{ "SerializeState": { "Mode": "Save", "Filename": "./states/EnRouteCare/Scenario3-InitialHemeostasis.json"} }</t>
@@ -1675,26 +1509,6 @@
  - Suction</t>
   </si>
   <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
-    "SupplementalSettings": { "Alarms" : { 
-    "HighPressureThreshold" : { "ScalarPressure": { "Value": 40, "Unit": "cmH2O" } },
-    "HighPressureCycleOption": "On",
-    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 9.6, "Unit": "L/min" } },
-    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 310, "Unit": "mL" } },
-    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 35, "Unit": "1/min" } } } } },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.5 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 30, "Unit": "cmH2O" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 25, "Unit": "1/min" } },
-  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
-  }}
-}</t>
-  </si>
-  <si>
     <t xml:space="preserve">Learning Objectives:
  - Assess baseline status
  - Recognize moderate ARDS
@@ -1765,8 +1579,8 @@
   </si>
   <si>
     <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On",
-    "SupplementalSettings": { "Alarms" : { 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } },
+    "SupplementalSettings": { "Connection": "On",  "Alarms" : { 
     "HighPressureThreshold" : { "ScalarPressure": { "Value": 35, "Unit": "cmH2O" } },
     "HighPressureCycleOption": "On",
     "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 11, "Unit": "L/min" } },
@@ -1779,6 +1593,192 @@
   "InspiratoryPressure": { "ScalarPressure": { "Value": 25, "Unit": "cmH2O" } },
   "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
   "RespirationRate": { "ScalarFrequency": { "Value": 10, "Unit": "1/min" } },
+  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, 
+    "SupplementalSettings": { "Connection": "On", "Alarms" : { 
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 28, "Unit": "cmH2O" } },
+    "HighPressureCycleOption": "On",
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 7.9, "Unit": "L/min" } },
+    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 365, "Unit": "mL" } },
+    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 33, "Unit": "1/min" } } } } },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.8, "Unit": "s" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 18, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 23, "Unit": "1/min" } },
+  "InspirationPatientTriggerFlow": { "ScalarVolumePerTime": { "Value": 1.0, "Unit": "L/min"  } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, 
+    "SupplementalSettings": { "Connection": "On", "Alarms" : { 
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 24, "Unit": "cmH2O" } },
+    "HighPressureCycleOption": "On",
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 8.4, "Unit": "L/min" } },
+    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 365, "Unit": "mL" } },
+    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 33, "Unit": "1/min" } } } } },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.8, "Unit": "s" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 14.2, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 10, "Unit": "1/min" } },
+  "InspirationPatientTriggerFlow": { "ScalarVolumePerTime": { "Value": 1.0, "Unit": "L/min"  } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, 
+    "SupplementalSettings": { "Connection": "On", "Alarms" : { 
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 40, "Unit": "cmH2O" } },
+    "HighPressureCycleOption": "On",
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 9.6, "Unit": "L/min" } },
+    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 310, "Unit": "mL" } },
+    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 35, "Unit": "1/min" } } } } },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.5 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 30, "Unit": "cmH2O" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 25, "Unit": "1/min" } },
+  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, 
+    "SupplementalSettings": { "Connection": "On", "Alarms" : { 
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 31, "Unit": "cmH2O" } },
+    "HighPressureCycleOption": "On",
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 7.3, "Unit": "L/min" } },
+    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 290, "Unit": "mL" } },
+    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 36, "Unit": "1/min" } } } } },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 42, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 26, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 376, "Unit": "mL" } },
+  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, 
+    "SupplementalSettings": { "Connection": "On", "Alarms" : { 
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 26, "Unit": "cmH2O" } },
+    "HighPressureCycleOption": "On",
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 7.5, "Unit": "L/min" } },
+    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 290, "Unit": "mL" } },
+    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 36, "Unit": "1/min" } } } } },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 42, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 12, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 376, "Unit": "mL" } },
+  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, 
+    "SupplementalSettings": { "Connection": "On",  "Alarms" : { 
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 37, "Unit": "cmH2O" } },
+    "HighPressureCycleOption": "On",
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 8.7, "Unit": "L/min" } },
+    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 360, "Unit": "mL" } },
+    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 34, "Unit": "1/min" } } } } },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 52, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 24, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 488, "Unit": "mL" } },
+  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, 
+    "SupplementalSettings": { "Connection": "On", "Alarms" : { 
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 33, "Unit": "cmH2O" } },
+    "HighPressureCycleOption": "On",
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 6.8, "Unit": "L/min" } },
+    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 330, "Unit": "mL" } },
+    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 30, "Unit": "1/min" } } } } },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 35, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.5 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.8, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 8, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 24, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 450, "Unit": "mL" } },
+   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, 
+    "SupplementalSettings": { "Connection": "On", "Alarms" : { 
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 50, "Unit": "cmH2O" } },
+    "HighPressureCycleOption": "On",
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 6.8, "Unit": "L/min" } },
+    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 490, "Unit": "mL" } },
+    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 24, "Unit": "1/min" } } } } },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 70, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 14, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 650, "Unit": "mL" } },
+  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, 
+    "SupplementalSettings": { "Connection": "On", "Alarms" : { 
+    "HighPressureThreshold" : { "ScalarPressure": { "Value": 38, "Unit": "cmH2O" } },
+    "HighPressureCycleOption": "On",
+    "LowMinuteVentilationThreshold" : { "ScalarVolumePerTime": { "Value": 10.4, "Unit": "L/min" } },
+    "LowTidalVolumeThreshold" : { "ScalarVolume": { "Value": 438, "Unit": "mL" } },
+    "HighRespiratoryRateThreshold" : { "ScalarFrequency": { "Value": 34, "Unit": "1/min" } } } } },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 60, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.62, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 24, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 584, "Unit": "mL" } },
   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
   }}
 }</t>
@@ -3185,7 +3185,7 @@
         <v>230</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G2" s="52"/>
       <c r="H2" s="52"/>
@@ -3344,7 +3344,7 @@
       <c r="E12" s="40"/>
       <c r="F12" s="40"/>
       <c r="G12" s="9" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="H12" s="17"/>
     </row>
@@ -3399,14 +3399,14 @@
         <v>1</v>
       </c>
       <c r="B16" s="40" t="s">
-        <v>275</v>
+        <v>359</v>
       </c>
       <c r="C16" s="54"/>
       <c r="D16" s="54"/>
       <c r="E16" s="54"/>
       <c r="F16" s="55"/>
       <c r="G16" s="9" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="H16" s="17"/>
     </row>
@@ -3625,7 +3625,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="40" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C27" s="40"/>
       <c r="D27" s="40"/>
@@ -3646,7 +3646,7 @@
       <c r="E28" s="40"/>
       <c r="F28" s="40"/>
       <c r="G28" s="9" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="H28" s="17"/>
     </row>
@@ -3655,7 +3655,7 @@
         <v>2</v>
       </c>
       <c r="B29" s="40" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C29" s="40"/>
       <c r="D29" s="40"/>
@@ -3676,7 +3676,7 @@
       <c r="E30" s="40"/>
       <c r="F30" s="40"/>
       <c r="G30" s="9" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="H30" s="17"/>
     </row>
@@ -3775,7 +3775,7 @@
         <v>27</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>28</v>
@@ -3788,7 +3788,7 @@
       </c>
       <c r="F35" s="10"/>
       <c r="G35" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H35" s="17"/>
     </row>
@@ -3841,7 +3841,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>32</v>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="F38" s="10"/>
       <c r="G38" s="12" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="H38" s="17"/>
     </row>
@@ -3881,7 +3881,7 @@
         <v>3</v>
       </c>
       <c r="B40" s="40" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C40" s="40"/>
       <c r="D40" s="40"/>
@@ -3902,7 +3902,7 @@
       <c r="E41" s="40"/>
       <c r="F41" s="40"/>
       <c r="G41" s="9" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="H41" s="17"/>
     </row>
@@ -3911,7 +3911,7 @@
         <v>3</v>
       </c>
       <c r="B42" s="40" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C42" s="40"/>
       <c r="D42" s="40"/>
@@ -4031,7 +4031,7 @@
         <v>27</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>28</v>
@@ -4044,7 +4044,7 @@
       </c>
       <c r="F48" s="10"/>
       <c r="G48" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H48" s="17"/>
     </row>
@@ -4183,7 +4183,7 @@
         <v>235</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="G2" s="52"/>
       <c r="H2" s="52"/>
@@ -4342,7 +4342,7 @@
       <c r="E12" s="40"/>
       <c r="F12" s="40"/>
       <c r="G12" s="9" t="s">
-        <v>356</v>
+        <v>347</v>
       </c>
       <c r="H12" s="17"/>
     </row>
@@ -4381,14 +4381,14 @@
         <v>1</v>
       </c>
       <c r="B15" s="53" t="s">
-        <v>364</v>
+        <v>355</v>
       </c>
       <c r="C15" s="54"/>
       <c r="D15" s="54"/>
       <c r="E15" s="54"/>
       <c r="F15" s="55"/>
       <c r="G15" s="9" t="s">
-        <v>363</v>
+        <v>354</v>
       </c>
       <c r="H15" s="17"/>
     </row>
@@ -4601,14 +4601,14 @@
         <v>2</v>
       </c>
       <c r="B26" s="40" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="C26" s="40"/>
       <c r="D26" s="40"/>
       <c r="E26" s="40"/>
       <c r="F26" s="40"/>
       <c r="G26" s="9" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="H26" s="17"/>
     </row>
@@ -4638,7 +4638,7 @@
       <c r="E28" s="40"/>
       <c r="F28" s="40"/>
       <c r="G28" s="9" t="s">
-        <v>354</v>
+        <v>346</v>
       </c>
       <c r="H28" s="17"/>
     </row>
@@ -4737,7 +4737,7 @@
         <v>27</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>28</v>
@@ -4750,7 +4750,7 @@
       </c>
       <c r="F33" s="10"/>
       <c r="G33" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H33" s="17"/>
     </row>
@@ -4798,7 +4798,7 @@
       <c r="E36" s="40"/>
       <c r="F36" s="40"/>
       <c r="G36" s="9" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="H36" s="17"/>
     </row>
@@ -4927,7 +4927,7 @@
         <v>27</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>28</v>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="F43" s="10"/>
       <c r="G43" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H43" s="17"/>
     </row>
@@ -5034,7 +5034,7 @@
         <v>235</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="G2" s="52"/>
       <c r="H2" s="52"/>
@@ -5193,7 +5193,7 @@
       <c r="E12" s="40"/>
       <c r="F12" s="40"/>
       <c r="G12" s="9" t="s">
-        <v>356</v>
+        <v>347</v>
       </c>
       <c r="H12" s="17"/>
     </row>
@@ -5248,14 +5248,14 @@
         <v>1</v>
       </c>
       <c r="B16" s="53" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="C16" s="54"/>
       <c r="D16" s="54"/>
       <c r="E16" s="54"/>
       <c r="F16" s="55"/>
       <c r="G16" s="9" t="s">
-        <v>357</v>
+        <v>348</v>
       </c>
       <c r="H16" s="17"/>
     </row>
@@ -5454,7 +5454,7 @@
         <v>2</v>
       </c>
       <c r="B26" s="40" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C26" s="40"/>
       <c r="D26" s="40"/>
@@ -5468,14 +5468,14 @@
         <v>2</v>
       </c>
       <c r="B27" s="40" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="C27" s="40"/>
       <c r="D27" s="40"/>
       <c r="E27" s="40"/>
       <c r="F27" s="40"/>
       <c r="G27" s="9" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="H27" s="17"/>
     </row>
@@ -5484,7 +5484,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="40" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C28" s="40"/>
       <c r="D28" s="40"/>
@@ -5505,7 +5505,7 @@
       <c r="E29" s="40"/>
       <c r="F29" s="40"/>
       <c r="G29" s="9" t="s">
-        <v>354</v>
+        <v>346</v>
       </c>
       <c r="H29" s="17"/>
     </row>
@@ -5604,7 +5604,7 @@
         <v>27</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>28</v>
@@ -5617,7 +5617,7 @@
       </c>
       <c r="F34" s="10"/>
       <c r="G34" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H34" s="17"/>
     </row>
@@ -5644,7 +5644,7 @@
         <v>3</v>
       </c>
       <c r="B36" s="40" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C36" s="40"/>
       <c r="D36" s="40"/>
@@ -5665,7 +5665,7 @@
       <c r="E37" s="40"/>
       <c r="F37" s="40"/>
       <c r="G37" s="9" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="H37" s="17"/>
     </row>
@@ -5674,7 +5674,7 @@
         <v>3</v>
       </c>
       <c r="B38" s="40" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C38" s="40"/>
       <c r="D38" s="40"/>
@@ -5794,7 +5794,7 @@
         <v>27</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>28</v>
@@ -5807,7 +5807,7 @@
       </c>
       <c r="F44" s="10"/>
       <c r="G44" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H44" s="17"/>
     </row>
@@ -5902,7 +5902,7 @@
         <v>240</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>353</v>
+        <v>345</v>
       </c>
       <c r="G2" s="52"/>
       <c r="H2" s="52"/>
@@ -6077,7 +6077,7 @@
       <c r="E13" s="40"/>
       <c r="F13" s="40"/>
       <c r="G13" s="9" t="s">
-        <v>358</v>
+        <v>349</v>
       </c>
       <c r="H13" s="17"/>
     </row>
@@ -6116,14 +6116,14 @@
         <v>1</v>
       </c>
       <c r="B16" s="40" t="s">
-        <v>252</v>
+        <v>357</v>
       </c>
       <c r="C16" s="40"/>
       <c r="D16" s="40"/>
       <c r="E16" s="40"/>
       <c r="F16" s="40"/>
       <c r="G16" s="9" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="H16" s="17"/>
     </row>
@@ -6363,7 +6363,7 @@
       <c r="E28" s="40"/>
       <c r="F28" s="40"/>
       <c r="G28" s="9" t="s">
-        <v>351</v>
+        <v>343</v>
       </c>
       <c r="H28" s="17"/>
     </row>
@@ -6386,7 +6386,7 @@
         <v>2</v>
       </c>
       <c r="B30" s="40" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="C30" s="40"/>
       <c r="D30" s="40"/>
@@ -6434,12 +6434,12 @@
         <v>50</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="E32" s="10"/>
       <c r="F32" s="10"/>
       <c r="G32" s="2" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="H32" s="17"/>
     </row>
@@ -6448,7 +6448,7 @@
         <v>27</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>28</v>
@@ -6461,7 +6461,7 @@
       </c>
       <c r="F33" s="10"/>
       <c r="G33" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H33" s="17"/>
     </row>
@@ -6509,7 +6509,7 @@
       <c r="E36" s="40"/>
       <c r="F36" s="40"/>
       <c r="G36" s="9" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="H36" s="17"/>
     </row>
@@ -6638,7 +6638,7 @@
         <v>27</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>28</v>
@@ -6651,7 +6651,7 @@
       </c>
       <c r="F43" s="10"/>
       <c r="G43" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H43" s="17"/>
     </row>
@@ -6746,7 +6746,7 @@
         <v>240</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>353</v>
+        <v>345</v>
       </c>
       <c r="G2" s="52"/>
       <c r="H2" s="52"/>
@@ -6921,7 +6921,7 @@
       <c r="E13" s="40"/>
       <c r="F13" s="40"/>
       <c r="G13" s="9" t="s">
-        <v>358</v>
+        <v>349</v>
       </c>
       <c r="H13" s="17"/>
     </row>
@@ -6976,14 +6976,14 @@
         <v>1</v>
       </c>
       <c r="B17" s="40" t="s">
-        <v>276</v>
+        <v>356</v>
       </c>
       <c r="C17" s="40"/>
       <c r="D17" s="40"/>
       <c r="E17" s="40"/>
       <c r="F17" s="40"/>
       <c r="G17" s="9" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="H17" s="17"/>
     </row>
@@ -7202,7 +7202,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="40" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C28" s="40"/>
       <c r="D28" s="40"/>
@@ -7223,7 +7223,7 @@
       <c r="E29" s="40"/>
       <c r="F29" s="40"/>
       <c r="G29" s="9" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="H29" s="17"/>
     </row>
@@ -7232,7 +7232,7 @@
         <v>2</v>
       </c>
       <c r="B30" s="40" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="C30" s="40"/>
       <c r="D30" s="40"/>
@@ -7246,7 +7246,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="40" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="C31" s="40"/>
       <c r="D31" s="40"/>
@@ -7294,12 +7294,12 @@
         <v>50</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
       <c r="G33" s="2" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="H33" s="17"/>
     </row>
@@ -7308,7 +7308,7 @@
         <v>27</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>28</v>
@@ -7321,7 +7321,7 @@
       </c>
       <c r="F34" s="10"/>
       <c r="G34" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H34" s="17"/>
     </row>
@@ -7348,7 +7348,7 @@
         <v>3</v>
       </c>
       <c r="B36" s="40" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="C36" s="40"/>
       <c r="D36" s="40"/>
@@ -7369,7 +7369,7 @@
       <c r="E37" s="40"/>
       <c r="F37" s="40"/>
       <c r="G37" s="9" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="H37" s="17"/>
     </row>
@@ -7378,7 +7378,7 @@
         <v>3</v>
       </c>
       <c r="B38" s="40" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="C38" s="40"/>
       <c r="D38" s="40"/>
@@ -7498,7 +7498,7 @@
         <v>27</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>28</v>
@@ -7511,7 +7511,7 @@
       </c>
       <c r="F44" s="10"/>
       <c r="G44" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H44" s="17"/>
     </row>
@@ -7611,7 +7611,7 @@
         <v>215</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="G2" s="52"/>
       <c r="H2" s="52"/>
@@ -7768,7 +7768,7 @@
       <c r="E12" s="40"/>
       <c r="F12" s="40"/>
       <c r="G12" s="9" t="s">
-        <v>362</v>
+        <v>353</v>
       </c>
       <c r="H12" s="9"/>
     </row>
@@ -7823,14 +7823,14 @@
         <v>1</v>
       </c>
       <c r="B16" s="40" t="s">
-        <v>326</v>
+        <v>364</v>
       </c>
       <c r="C16" s="54"/>
       <c r="D16" s="54"/>
       <c r="E16" s="54"/>
       <c r="F16" s="55"/>
       <c r="G16" s="9" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="H16" s="9"/>
     </row>
@@ -7885,7 +7885,7 @@
         <v>50</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
@@ -8070,7 +8070,7 @@
       <c r="E28" s="40"/>
       <c r="F28" s="40"/>
       <c r="G28" s="9" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="H28" s="9"/>
     </row>
@@ -8086,7 +8086,7 @@
       <c r="E29" s="40"/>
       <c r="F29" s="40"/>
       <c r="G29" s="9" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="H29" s="9"/>
     </row>
@@ -8361,7 +8361,7 @@
         <v>27</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>28</v>
@@ -8374,7 +8374,7 @@
       </c>
       <c r="F43" s="10"/>
       <c r="G43" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H43" s="17"/>
     </row>
@@ -8415,14 +8415,14 @@
         <v>3</v>
       </c>
       <c r="B46" s="40" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="C46" s="40"/>
       <c r="D46" s="40"/>
       <c r="E46" s="40"/>
       <c r="F46" s="40"/>
       <c r="G46" s="9" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="H46" s="17"/>
     </row>
@@ -8553,14 +8553,14 @@
         <v>4</v>
       </c>
       <c r="B53" s="40" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="C53" s="40"/>
       <c r="D53" s="40"/>
       <c r="E53" s="40"/>
       <c r="F53" s="40"/>
       <c r="G53" s="9" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="H53" s="17"/>
     </row>
@@ -8848,7 +8848,7 @@
         <v>215</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="G2" s="52"/>
       <c r="H2" s="52"/>
@@ -9005,7 +9005,7 @@
       <c r="E12" s="40"/>
       <c r="F12" s="40"/>
       <c r="G12" s="9" t="s">
-        <v>362</v>
+        <v>353</v>
       </c>
       <c r="H12" s="9"/>
     </row>
@@ -9060,14 +9060,14 @@
         <v>1</v>
       </c>
       <c r="B16" s="40" t="s">
-        <v>326</v>
+        <v>364</v>
       </c>
       <c r="C16" s="54"/>
       <c r="D16" s="54"/>
       <c r="E16" s="54"/>
       <c r="F16" s="55"/>
       <c r="G16" s="9" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="H16" s="9"/>
     </row>
@@ -9122,7 +9122,7 @@
         <v>50</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
@@ -9286,7 +9286,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="40" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C27" s="40"/>
       <c r="D27" s="40"/>
@@ -9307,7 +9307,7 @@
       <c r="E28" s="54"/>
       <c r="F28" s="55"/>
       <c r="G28" s="9" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="H28" s="9"/>
     </row>
@@ -9323,7 +9323,7 @@
       <c r="E29" s="40"/>
       <c r="F29" s="40"/>
       <c r="G29" s="9" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="H29" s="9"/>
     </row>
@@ -9348,7 +9348,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="40" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C31" s="40"/>
       <c r="D31" s="40"/>
@@ -9598,7 +9598,7 @@
         <v>27</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>28</v>
@@ -9611,7 +9611,7 @@
       </c>
       <c r="F43" s="10"/>
       <c r="G43" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H43" s="17"/>
     </row>
@@ -9638,7 +9638,7 @@
         <v>3</v>
       </c>
       <c r="B45" s="40" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C45" s="40"/>
       <c r="D45" s="40"/>
@@ -9652,14 +9652,14 @@
         <v>3</v>
       </c>
       <c r="B46" s="40" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="C46" s="40"/>
       <c r="D46" s="40"/>
       <c r="E46" s="40"/>
       <c r="F46" s="40"/>
       <c r="G46" s="9" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="H46" s="17"/>
     </row>
@@ -9790,14 +9790,14 @@
         <v>4</v>
       </c>
       <c r="B53" s="40" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="C53" s="40"/>
       <c r="D53" s="40"/>
       <c r="E53" s="40"/>
       <c r="F53" s="40"/>
       <c r="G53" s="9" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="H53" s="17"/>
     </row>
@@ -9806,7 +9806,7 @@
         <v>4</v>
       </c>
       <c r="B54" s="40" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C54" s="40"/>
       <c r="D54" s="40"/>
@@ -10083,7 +10083,7 @@
         <v>219</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="G2" s="52"/>
       <c r="H2" s="52"/>
@@ -10244,7 +10244,7 @@
       <c r="E12" s="40"/>
       <c r="F12" s="40"/>
       <c r="G12" s="9" t="s">
-        <v>361</v>
+        <v>352</v>
       </c>
       <c r="H12" s="17"/>
     </row>
@@ -10281,14 +10281,14 @@
         <v>1</v>
       </c>
       <c r="B15" s="53" t="s">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C15" s="54"/>
       <c r="D15" s="54"/>
       <c r="E15" s="54"/>
       <c r="F15" s="55"/>
       <c r="G15" s="9" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="H15" s="17"/>
     </row>
@@ -10594,7 +10594,7 @@
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
       <c r="G31" s="2" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="H31" s="17"/>
     </row>
@@ -10701,14 +10701,14 @@
         <v>3</v>
       </c>
       <c r="B37" s="53" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="C37" s="54"/>
       <c r="D37" s="54"/>
       <c r="E37" s="54"/>
       <c r="F37" s="55"/>
       <c r="G37" s="9" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="H37" s="17"/>
     </row>
@@ -10945,7 +10945,7 @@
         <v>219</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="G2" s="52"/>
       <c r="H2" s="52"/>
@@ -11106,7 +11106,7 @@
       <c r="E12" s="40"/>
       <c r="F12" s="40"/>
       <c r="G12" s="9" t="s">
-        <v>361</v>
+        <v>352</v>
       </c>
       <c r="H12" s="17"/>
     </row>
@@ -11143,14 +11143,14 @@
         <v>1</v>
       </c>
       <c r="B15" s="40" t="s">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C15" s="40"/>
       <c r="D15" s="40"/>
       <c r="E15" s="40"/>
       <c r="F15" s="40"/>
       <c r="G15" s="9" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="H15" s="17"/>
     </row>
@@ -11347,7 +11347,7 @@
         <v>2</v>
       </c>
       <c r="B25" s="40" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C25" s="40"/>
       <c r="D25" s="40"/>
@@ -11368,7 +11368,7 @@
       <c r="E26" s="40"/>
       <c r="F26" s="40"/>
       <c r="G26" s="9" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="H26" s="9"/>
     </row>
@@ -11391,7 +11391,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="40" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="C28" s="40"/>
       <c r="D28" s="40"/>
@@ -11456,7 +11456,7 @@
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
       <c r="G31" s="2" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="H31" s="17"/>
     </row>
@@ -11563,14 +11563,14 @@
         <v>3</v>
       </c>
       <c r="B37" s="53" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="C37" s="54"/>
       <c r="D37" s="54"/>
       <c r="E37" s="54"/>
       <c r="F37" s="55"/>
       <c r="G37" s="9" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="H37" s="17"/>
     </row>
@@ -11579,7 +11579,7 @@
         <v>3</v>
       </c>
       <c r="B38" s="40" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="C38" s="40"/>
       <c r="D38" s="40"/>
@@ -12821,7 +12821,7 @@
         <v>224</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="G2" s="52"/>
       <c r="H2" s="52"/>
@@ -24172,7 +24172,7 @@
       <c r="E13" s="40"/>
       <c r="F13" s="40"/>
       <c r="G13" s="19" t="s">
-        <v>360</v>
+        <v>351</v>
       </c>
       <c r="H13" s="17"/>
       <c r="I13" s="13"/>
@@ -27275,14 +27275,14 @@
         <v>1</v>
       </c>
       <c r="B17" s="40" t="s">
-        <v>316</v>
+        <v>362</v>
       </c>
       <c r="C17" s="40"/>
       <c r="D17" s="40"/>
       <c r="E17" s="40"/>
       <c r="F17" s="40"/>
       <c r="G17" s="19" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="H17" s="17"/>
       <c r="I17" s="13"/>
@@ -31565,7 +31565,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="40" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="C28" s="40"/>
       <c r="D28" s="40"/>
@@ -32602,7 +32602,7 @@
       <c r="E29" s="40"/>
       <c r="F29" s="40"/>
       <c r="G29" s="19" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="H29" s="17"/>
       <c r="I29" s="13"/>
@@ -33627,7 +33627,7 @@
         <v>2</v>
       </c>
       <c r="B30" s="40" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="C30" s="40"/>
       <c r="D30" s="40"/>
@@ -33635,7 +33635,7 @@
       <c r="F30" s="40"/>
       <c r="G30" s="19"/>
       <c r="H30" s="17" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="I30" s="13"/>
       <c r="J30" s="13"/>
@@ -38805,7 +38805,7 @@
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
       <c r="G35" s="20" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="H35" s="17"/>
     </row>
@@ -38902,7 +38902,7 @@
         <v>27</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>28</v>
@@ -38915,7 +38915,7 @@
       </c>
       <c r="F40" s="10"/>
       <c r="G40" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H40" s="17"/>
     </row>
@@ -40025,24 +40025,24 @@
     </row>
     <row r="45" spans="1:1024" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="36" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="E45" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F45" s="2"/>
       <c r="G45" s="2" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="H45" s="36" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
     </row>
     <row r="46" spans="1:1024" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
@@ -41084,7 +41084,7 @@
         <v>3</v>
       </c>
       <c r="B47" s="40" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="C47" s="40"/>
       <c r="D47" s="40"/>
@@ -42114,14 +42114,14 @@
         <v>3</v>
       </c>
       <c r="B48" s="40" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="C48" s="40"/>
       <c r="D48" s="40"/>
       <c r="E48" s="40"/>
       <c r="F48" s="40"/>
       <c r="G48" s="19" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="H48" s="17"/>
       <c r="I48" s="13"/>
@@ -45257,24 +45257,24 @@
     </row>
     <row r="53" spans="1:1024" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" s="36" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="E53" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F53" s="2"/>
       <c r="G53" s="2" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="H53" s="36" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
     </row>
     <row r="54" spans="1:1024" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
@@ -46316,14 +46316,14 @@
         <v>4</v>
       </c>
       <c r="B55" s="40" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="C55" s="40"/>
       <c r="D55" s="40"/>
       <c r="E55" s="40"/>
       <c r="F55" s="40"/>
       <c r="G55" s="19" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="H55" s="17"/>
       <c r="I55" s="13"/>
@@ -47348,7 +47348,7 @@
         <v>4</v>
       </c>
       <c r="B56" s="40" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="C56" s="40"/>
       <c r="D56" s="40"/>
@@ -50470,7 +50470,7 @@
         <v>27</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>28</v>
@@ -50483,7 +50483,7 @@
       </c>
       <c r="F60" s="10"/>
       <c r="G60" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H60" s="17"/>
     </row>
@@ -50511,32 +50511,30 @@
     </row>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="B56:F56"/>
-    <mergeCell ref="B57:F57"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B56:F56"/>
+    <mergeCell ref="B57:F57"/>
     <mergeCell ref="G6:H9"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="B55:F55"/>
     <mergeCell ref="B17:F17"/>
@@ -50550,6 +50548,8 @@
     <mergeCell ref="B46:F46"/>
     <mergeCell ref="B47:F47"/>
     <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B33:F33"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -50605,7 +50605,7 @@
         <v>224</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="G2" s="52"/>
       <c r="H2" s="52"/>
@@ -50780,7 +50780,7 @@
       <c r="E13" s="40"/>
       <c r="F13" s="40"/>
       <c r="G13" s="19" t="s">
-        <v>360</v>
+        <v>351</v>
       </c>
       <c r="H13" s="17"/>
     </row>
@@ -50835,14 +50835,14 @@
         <v>1</v>
       </c>
       <c r="B17" s="40" t="s">
-        <v>316</v>
+        <v>362</v>
       </c>
       <c r="C17" s="40"/>
       <c r="D17" s="40"/>
       <c r="E17" s="40"/>
       <c r="F17" s="40"/>
       <c r="G17" s="19" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="H17" s="17"/>
     </row>
@@ -51061,7 +51061,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="40" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C28" s="40"/>
       <c r="D28" s="40"/>
@@ -51082,7 +51082,7 @@
       <c r="E29" s="40"/>
       <c r="F29" s="40"/>
       <c r="G29" s="19" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="H29" s="17"/>
     </row>
@@ -51098,7 +51098,7 @@
       <c r="E30" s="40"/>
       <c r="F30" s="40"/>
       <c r="G30" s="19" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="H30" s="17"/>
     </row>
@@ -51107,7 +51107,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="40" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="C31" s="40"/>
       <c r="D31" s="40"/>
@@ -51115,7 +51115,7 @@
       <c r="F31" s="40"/>
       <c r="G31" s="19"/>
       <c r="H31" s="17" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="121.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -51189,7 +51189,7 @@
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
       <c r="G35" s="20" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="H35" s="17"/>
     </row>
@@ -51286,7 +51286,7 @@
         <v>27</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>28</v>
@@ -51299,7 +51299,7 @@
       </c>
       <c r="F40" s="10"/>
       <c r="G40" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H40" s="17"/>
     </row>
@@ -51393,24 +51393,24 @@
     </row>
     <row r="45" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="36" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="E45" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F45" s="2"/>
       <c r="G45" s="2" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="H45" s="36" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
@@ -51436,7 +51436,7 @@
         <v>3</v>
       </c>
       <c r="B47" s="40" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C47" s="40"/>
       <c r="D47" s="40"/>
@@ -51450,14 +51450,14 @@
         <v>3</v>
       </c>
       <c r="B48" s="40" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="C48" s="40"/>
       <c r="D48" s="40"/>
       <c r="E48" s="40"/>
       <c r="F48" s="40"/>
       <c r="G48" s="19" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="H48" s="17"/>
     </row>
@@ -51545,24 +51545,24 @@
     </row>
     <row r="53" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" s="36" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="E53" s="10" t="s">
         <v>29</v>
       </c>
       <c r="F53" s="2"/>
       <c r="G53" s="2" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="H53" s="36" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
     </row>
     <row r="54" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
@@ -51588,14 +51588,14 @@
         <v>4</v>
       </c>
       <c r="B55" s="40" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="C55" s="40"/>
       <c r="D55" s="40"/>
       <c r="E55" s="40"/>
       <c r="F55" s="40"/>
       <c r="G55" s="19" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="H55" s="17"/>
     </row>
@@ -51604,7 +51604,7 @@
         <v>4</v>
       </c>
       <c r="B56" s="40" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C56" s="40"/>
       <c r="D56" s="40"/>
@@ -51678,7 +51678,7 @@
         <v>27</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>28</v>
@@ -51691,7 +51691,7 @@
       </c>
       <c r="F60" s="10"/>
       <c r="G60" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H60" s="17"/>
     </row>
@@ -51814,7 +51814,7 @@
         <v>225</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="G2" s="52"/>
       <c r="H2" s="52"/>
@@ -51989,7 +51989,7 @@
       <c r="E13" s="40"/>
       <c r="F13" s="40"/>
       <c r="G13" s="9" t="s">
-        <v>356</v>
+        <v>347</v>
       </c>
       <c r="H13" s="17"/>
     </row>
@@ -52044,14 +52044,14 @@
         <v>1</v>
       </c>
       <c r="B17" s="40" t="s">
-        <v>250</v>
+        <v>361</v>
       </c>
       <c r="C17" s="54"/>
       <c r="D17" s="54"/>
       <c r="E17" s="54"/>
       <c r="F17" s="55"/>
       <c r="G17" s="9" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="H17" s="17"/>
     </row>
@@ -52291,7 +52291,7 @@
       <c r="E29" s="40"/>
       <c r="F29" s="40"/>
       <c r="G29" s="9" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="H29" s="17"/>
     </row>
@@ -52464,7 +52464,7 @@
         <v>27</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>28</v>
@@ -52477,7 +52477,7 @@
       </c>
       <c r="F38" s="10"/>
       <c r="G38" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H38" s="17"/>
     </row>
@@ -52569,7 +52569,7 @@
       <c r="E43" s="40"/>
       <c r="F43" s="40"/>
       <c r="G43" s="9" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="H43" s="17"/>
     </row>
@@ -52585,7 +52585,7 @@
       <c r="E44" s="40"/>
       <c r="F44" s="40"/>
       <c r="G44" s="9" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="H44" s="17" t="s">
         <v>91</v>
@@ -52758,7 +52758,7 @@
         <v>27</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>28</v>
@@ -52771,7 +52771,7 @@
       </c>
       <c r="F53" s="10"/>
       <c r="G53" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H53" s="17"/>
     </row>
@@ -52912,7 +52912,7 @@
         <v>230</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="G2" s="52"/>
       <c r="H2" s="52"/>
@@ -53071,7 +53071,7 @@
       <c r="E12" s="40"/>
       <c r="F12" s="40"/>
       <c r="G12" s="9" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="H12" s="17"/>
     </row>
@@ -53110,14 +53110,14 @@
         <v>1</v>
       </c>
       <c r="B15" s="40" t="s">
-        <v>251</v>
+        <v>360</v>
       </c>
       <c r="C15" s="54"/>
       <c r="D15" s="54"/>
       <c r="E15" s="54"/>
       <c r="F15" s="55"/>
       <c r="G15" s="9" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="H15" s="17"/>
     </row>
@@ -53357,7 +53357,7 @@
       <c r="E27" s="40"/>
       <c r="F27" s="40"/>
       <c r="G27" s="9" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="H27" s="17"/>
     </row>
@@ -53387,7 +53387,7 @@
       <c r="E29" s="40"/>
       <c r="F29" s="40"/>
       <c r="G29" s="9" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="H29" s="17"/>
     </row>
@@ -53486,7 +53486,7 @@
         <v>27</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>28</v>
@@ -53499,7 +53499,7 @@
       </c>
       <c r="F34" s="10"/>
       <c r="G34" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H34" s="17"/>
     </row>
@@ -53552,7 +53552,7 @@
         <v>37</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>32</v>
@@ -53565,7 +53565,7 @@
       </c>
       <c r="F37" s="10"/>
       <c r="G37" s="12" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="H37" s="17"/>
     </row>
@@ -53613,7 +53613,7 @@
       <c r="E40" s="40"/>
       <c r="F40" s="40"/>
       <c r="G40" s="9" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="H40" s="17"/>
     </row>
@@ -53742,7 +53742,7 @@
         <v>27</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>28</v>
@@ -53755,7 +53755,7 @@
       </c>
       <c r="F47" s="10"/>
       <c r="G47" s="12" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H47" s="17"/>
     </row>

</xml_diff>